<commit_message>
sims: pre-send audit FIX — v5 Scenario B13/B15 spoof (skeptic/Opus)
Auditor (pre-send red-team) found a hard FLAG-SPOOF: Scenario_calc B13
(BASE) and B15 (RESTAKED) had broken formulas computing -66.26%/-67.76%
(sign-flipped) vs the report's +40.2%/+50.2% — the exact cells the report
cites and invites Varun to open. FIXED: B13=B9+B10+B11+B12, B15=B13+B14 ->
40.24%/50.24%. Grids (Exhibits A/B) were correct; v3/v4 unaffected.
NITs fixed: Financing row added to Exhibit C (tie-out); Q2 "widens
profitable region" softened (no shown cell flips). Report re-rendered.
Verdict after fixes: SAFE TO SEND. NON-CORE.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cs1cJ4yQMcmxqbEVrDpqHd
</commit_message>
<xml_diff>
--- a/sims/temporal_lp_economics_MODEL_v5_options_seller.xlsx
+++ b/sims/temporal_lp_economics_MODEL_v5_options_seller.xlsx
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>B8+B9+B10+B11</f>
+        <f>B9+B10+B11+B12</f>
         <v/>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>B12+B13</f>
+        <f>B13+B14</f>
         <v/>
       </c>
     </row>

</xml_diff>